<commit_message>
docs: add video link and update registration data
- Add YouTube video link for 2025/12/06 macro reading group session
- Update reading group registration spreadsheet

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/members/Reading Group Registration (Responses).xlsx
+++ b/members/Reading Group Registration (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="87">
   <si>
     <t>Timestamp</t>
   </si>
@@ -214,9 +214,6 @@
     <t>https://www.facebook.com/duong.tung.bui.7976/</t>
   </si>
   <si>
-    <t>Foreign Trade University - Hanoi campus</t>
-  </si>
-  <si>
     <t>University of Western Ontario, Canada</t>
   </si>
   <si>
@@ -254,6 +251,27 @@
   </si>
   <si>
     <t>Econometrics</t>
+  </si>
+  <si>
+    <t>Đoàn Mạnh Đức</t>
+  </si>
+  <si>
+    <t>manhduc.doan03@gmail.com</t>
+  </si>
+  <si>
+    <t>manhducdoan.github.io</t>
+  </si>
+  <si>
+    <t>Microeconomics, Econometrics, Labor, Education, Development, IO, Public economics, Economic history, Political economy</t>
+  </si>
+  <si>
+    <t>Connecting to Power: Political Connections, Innovation, and Firm Dynamics</t>
+  </si>
+  <si>
+    <t>D70, O3, O4</t>
+  </si>
+  <si>
+    <t>Microeconomics, Macroeconomics, Political economy</t>
   </si>
 </sst>
 </file>
@@ -410,7 +428,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q9" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q10" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="17">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Full name" id="2"/>
@@ -951,19 +969,19 @@
         <v>50</v>
       </c>
       <c r="G8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="J8" s="7" t="s">
+      <c r="K8" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>24</v>
@@ -974,19 +992,19 @@
         <v>46109.90441265046</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>38</v>
@@ -998,25 +1016,72 @@
         <v>33</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>54</v>
       </c>
       <c r="M9" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="N9" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="7" t="s">
+      <c r="O9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="P9" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>80</v>
       </c>
       <c r="Q9" s="9">
         <v>46165.0</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="6">
+        <v>46114.5857575</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q10" s="9">
+        <v>46137.0</v>
       </c>
     </row>
   </sheetData>
@@ -1027,10 +1092,11 @@
     <hyperlink r:id="rId4" ref="E8"/>
     <hyperlink r:id="rId5" ref="D9"/>
     <hyperlink r:id="rId6" ref="E9"/>
+    <hyperlink r:id="rId7" ref="D10"/>
   </hyperlinks>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId8"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deploying to gh-pages from @ syve-econ/syve-econ.github.io@45f393bee464a2be73cdb710f846077ec3a14ec0 🚀
</commit_message>
<xml_diff>
--- a/members/Reading Group Registration (Responses).xlsx
+++ b/members/Reading Group Registration (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="87">
   <si>
     <t>Timestamp</t>
   </si>
@@ -214,9 +214,6 @@
     <t>https://www.facebook.com/duong.tung.bui.7976/</t>
   </si>
   <si>
-    <t>Foreign Trade University - Hanoi campus</t>
-  </si>
-  <si>
     <t>University of Western Ontario, Canada</t>
   </si>
   <si>
@@ -254,6 +251,27 @@
   </si>
   <si>
     <t>Econometrics</t>
+  </si>
+  <si>
+    <t>Đoàn Mạnh Đức</t>
+  </si>
+  <si>
+    <t>manhduc.doan03@gmail.com</t>
+  </si>
+  <si>
+    <t>manhducdoan.github.io</t>
+  </si>
+  <si>
+    <t>Microeconomics, Econometrics, Labor, Education, Development, IO, Public economics, Economic history, Political economy</t>
+  </si>
+  <si>
+    <t>Connecting to Power: Political Connections, Innovation, and Firm Dynamics</t>
+  </si>
+  <si>
+    <t>D70, O3, O4</t>
+  </si>
+  <si>
+    <t>Microeconomics, Macroeconomics, Political economy</t>
   </si>
 </sst>
 </file>
@@ -410,7 +428,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q9" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Q10" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="17">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Full name" id="2"/>
@@ -951,19 +969,19 @@
         <v>50</v>
       </c>
       <c r="G8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="J8" s="7" t="s">
+      <c r="K8" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>24</v>
@@ -974,19 +992,19 @@
         <v>46109.90441265046</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>38</v>
@@ -998,25 +1016,72 @@
         <v>33</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>54</v>
       </c>
       <c r="M9" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="N9" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="7" t="s">
+      <c r="O9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="P9" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>80</v>
       </c>
       <c r="Q9" s="9">
         <v>46165.0</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="6">
+        <v>46114.5857575</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q10" s="9">
+        <v>46137.0</v>
       </c>
     </row>
   </sheetData>
@@ -1027,10 +1092,11 @@
     <hyperlink r:id="rId4" ref="E8"/>
     <hyperlink r:id="rId5" ref="D9"/>
     <hyperlink r:id="rId6" ref="E9"/>
+    <hyperlink r:id="rId7" ref="D10"/>
   </hyperlinks>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId8"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>